<commit_message>
chore: release v1.7.64 - sync workspace and business csv import
</commit_message>
<xml_diff>
--- a/docs/导入中心Excel完整示例.xlsx
+++ b/docs/导入中心Excel完整示例.xlsx
@@ -7,8 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="统一知识与报价导入模板" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段说明" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="枚举参考" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,11 +416,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T5"/>
+  <dimension ref="A1:T10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -427,8 +429,8 @@
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
@@ -706,15 +708,19 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>英译法普通商务资料报价</t>
+          <t>英译法能力说明</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>英译法普通商务资料按220元/千字报价，最低收费300元。</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>可承接英译法普通商务资料，支持标准译审流程和按需润色。</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>能力知识</t>
+        </is>
+      </c>
       <c r="D5" t="n">
         <v>0</v>
       </c>
@@ -735,51 +741,333 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
+        <v>80</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>能力,英译法</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>价格异议案例</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>客户质疑价格高，销售先解释译审流程和交付保障，再补充历史交付经验，最终推进成交。</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>案例</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>翻译</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>普通资料</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>重点客户</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>65</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>案例,价格异议</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>询价回复邮件模板</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>您好，请您先发送需翻译文件，并说明语种、用途、交付时间和质量要求，我们收到后尽快评估报价。</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>邮件模板</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>翻译</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>普通资料</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="n">
+        <v>70</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>邮件模板,询价</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1000中文字符定义</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1000中文字符通常指中文原文字符数量，用于按千字计价的翻译报价口径。</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>名词定义</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>翻译</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>普通资料</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="n">
+        <v>55</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>定义,报价口径</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>英译法普通商务资料报价</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>英译法普通商务资料按220元/千字报价，最低收费300元。</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>翻译</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>英译法</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>普通资料</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="n">
         <v>95</v>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>高</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>2030-12-31</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>每千中文字符</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>CNY</t>
         </is>
       </c>
-      <c r="O5" t="n">
+      <c r="O9" t="n">
         <v>220</v>
       </c>
-      <c r="P5" t="n">
+      <c r="P9" t="n">
         <v>220</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="Q9" t="n">
         <v>300</v>
       </c>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr">
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr">
         <is>
           <t>不含税</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="T9" t="inlineStr">
         <is>
           <t>结构化报价</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>邮件询价整理</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>客户邮件询问英译法报价和交期，需先确认文件字数、用途、交付时间和是否需要盖章。</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>FAQ常见问答</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>翻译</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>英译法</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>认证/盖章文件</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>普通客户</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>72</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>邮件,询价整理</t>
         </is>
       </c>
     </row>
@@ -794,11 +1082,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="96" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -816,60 +1104,2374 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>统一模板</t>
+          <t>统一模板适用范围</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>该模板同时支持 7 类业务知识和结构化报价规则，无需先选择导入类型。</t>
+          <t>同一份模板同时支持 FAQ常见问答、流程规则、能力知识、案例、邮件模板、名词定义、报价限制条件，以及结构化报价规则。</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>知识分类</t>
+          <t>普通知识导入规则</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>除结构化报价规则外，其余业务知识必须填写知识分类。</t>
+          <t>普通业务知识必须填写知识分类；系统会根据知识分类自动映射到底层 knowledge_type 和 chunk_type。</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>结构化报价规则</t>
+          <t>结构化报价规则导入规则</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>结构化报价规则行的知识分类留空，填写价格、单位、币种、生效时间和失效时间等字段。</t>
+          <t>结构化报价规则行的知识分类留空，同时补齐价格、单位、币种、生效日期、失效日期等字段。</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>切分</t>
+          <t>切分规则</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>切分=1 时会调用 LLM 自动拆成多条草稿 chunk；结构化报价规则固定按单条导入。</t>
+          <t>切分=1 会调用 LLM 自动拆成多条草稿切片；结构化报价规则固定按单条导入。</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>审核发布</t>
+          <t>审核发布规则</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>所有导入结果先进入 draft，后续仍需提交审核、审核同意和发布门禁。</t>
+          <t>所有导入结果先进入 draft，仍需提交审核、审核同意并通过发布门禁后才能进入正式检索。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>样例使用方式</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>模板首个工作表中的示例行可直接另存为内部样例，删除示例后再填正式数据。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="33" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>字段</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>是否必填</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>适用范围</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>填写说明</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>示例</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>标题</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>全部知识</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>建议写成可被审核人快速判断用途的主题，避免过短或过泛。</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>翻译下单流程</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>内容</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>全部知识</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>填写可复用的业务说明、流程、问答、模板或规则正文。</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>收文件、确认语种用途、评估报价交期、付款立项、译审交付。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>知识分类</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>普通知识必填；结构化报价留空</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>FAQ/流程/能力/案例/邮件模板/名词定义/报价限制条件</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>统一模板用它判断落入哪类知识；结构化报价规则行请保持留空。</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>流程规则</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>切分</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>全部知识</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>填 1 时会调用 LLM 按业务知识点拆成多条草稿切片；填 0 或留空则按单条导入。</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>服务</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>建议填写</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>全部知识</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>用于限定业务线，常见值：翻译、印刷、同传、多媒体译制、展台搭建、礼品、通用。</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>翻译</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>按需填写</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>语言相关知识或报价</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>建议使用系统标准值，例如中译英、英译法、英译中。</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>英译法</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>服务范围</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>按需填写</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>全部知识</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>限定资料范围，例如普通资料、法律资料、认证/盖章文件。</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>普通资料</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>客户层级</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>按需填写</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>全部知识</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>用于限定知识适用对象，例如普通客户、重点客户、VIP客户。</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>重点客户</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>优先级</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>全部知识</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>数值越大代表排序时越靠前，建议 1-100。</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>风险等级</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>建议填写</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>全部知识</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>低/中/高；涉及报价承诺、限制条件、例外说明时建议填高。</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>生效日期</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>结构化报价建议填写</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>结构化报价规则</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>价格开始生效日期，支持 yyyy-mm-dd。</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>失效日期</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>结构化报价建议填写</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>结构化报价规则</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>价格失效日期，支持 yyyy-mm-dd。</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2030-12-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>单位</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>结构化报价建议填写</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>结构化报价规则</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>建议使用模板示例口径，例如每千中文字符、每项目、每小时。</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>每千中文字符</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>币种</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>结构化报价建议填写</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>结构化报价规则</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>如 CNY、USD。</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>价格</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>结构化报价建议填写</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>结构化报价规则</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>最低价格或单价；若只有一个价格，最高价格可与之相同或留空。</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>最高价格</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>结构化报价规则</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>用于价格区间上限；单点价格可留空或与价格相同。</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>最低收费</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>按需填写</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>结构化报价规则</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>项目低于最低收费时按该金额执行。</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>加急倍率</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>按需填写</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>结构化报价规则</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>只写明确可执行的倍率；不确定时应改写为报价限制条件。</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>税费</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>按需填写</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>结构化报价规则</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>记录含税/不含税、发票要求等。</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>不含税</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>标签</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>全部知识</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>多个标签用逗号分隔，方便后续筛选和审核。</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>流程,下单</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D77"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>字段</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>编码</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>显示值</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>知识分类</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>pricing_constraint</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>报价限制条件</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>统一模板里普通知识必填；结构化报价规则留空。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>知识分类</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>capability</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>能力知识</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>统一模板里普通知识必填；结构化报价规则留空。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>知识分类</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>流程规则</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>统一模板里普通知识必填；结构化报价规则留空。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>知识分类</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>faq</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>FAQ常见问答</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>统一模板里普通知识必填；结构化报价规则留空。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>知识分类</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>example</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>案例</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>统一模板里普通知识必填；结构化报价规则留空。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>知识分类</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>email_template</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>邮件模板</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>统一模板里普通知识必填；结构化报价规则留空。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>知识分类</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>definition</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>名词定义</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>统一模板里普通知识必填；结构化报价规则留空。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>服务</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>translation</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>翻译</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>用于限定业务线，推荐直接使用系统标准值。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>服务</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>printing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>印刷</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>用于限定业务线，推荐直接使用系统标准值。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>服务</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>interpretation</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>同传</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>用于限定业务线，推荐直接使用系统标准值。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>服务</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>multimedia</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>多媒体译制</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>用于限定业务线，推荐直接使用系统标准值。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>服务</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>exhibition</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>展台搭建</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>用于限定业务线，推荐直接使用系统标准值。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>服务</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>gifts</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>礼品</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>用于限定业务线，推荐直接使用系统标准值。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>服务</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>通用</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>用于限定业务线，推荐直接使用系统标准值。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>en-&gt;fr</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>英译法</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>en-&gt;zh</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>英译中</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>zh-&gt;en</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>中译英</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>en-&gt;ru</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>英译俄</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ja-&gt;zh</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>日译中</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ko-&gt;zh</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>韩译中</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>zh-&gt;ja</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>中译日</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>fr-&gt;zh</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>法译中</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>zh-&gt;fr</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>中译法</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>de-&gt;zh</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>德译中</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>zh-&gt;de</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>中译德</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ru-&gt;zh</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>俄译中</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>zh-&gt;ru</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>中译俄</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>zh-&gt;ko</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>中译韩</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>it-&gt;zh</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>意译中</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>zh-&gt;it</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>中译意</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>es-&gt;zh</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>西译中</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>zh-&gt;es</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>中译西</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ar-&gt;zh</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>阿译中</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>zh-&gt;ar</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>中译阿</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>da-&gt;zh</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>丹麦语译中</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>zh-&gt;da</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>中译丹麦语</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>pt-&gt;zh</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>葡译中</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>zh-&gt;pt</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>中译葡</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>nl-&gt;zh</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>荷译中</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>zh-&gt;nl</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>中译荷</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>sv-&gt;zh</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>瑞典语译中</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>zh-&gt;sv</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>中译瑞典语</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>no-&gt;zh</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>挪威语译中</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>zh-&gt;no</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>中译挪威语</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>el-&gt;zh</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>希腊语译中</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>zh-&gt;el</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>中译希腊语</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>tr-&gt;zh</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>土耳其语译中</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>zh-&gt;tr</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>中译土耳其语</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>fr-&gt;en</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>法译英</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>de-&gt;en</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>德译英</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>en-&gt;de</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>英译德</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>en-&gt;ja</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>英译日</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>ja-&gt;en</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>日译英</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>语种</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>en-&gt;en</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>英文润稿</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>只在与语言方向强相关的知识或报价里填写。</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>服务范围</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>普通资料</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>限定资料类型、项目范围或场景边界。</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>服务范围</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>medical</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>医学资料</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>限定资料类型、项目范围或场景边界。</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>服务范围</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>legal</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>法律资料</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>限定资料类型、项目范围或场景边界。</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>服务范围</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>technical</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>技术资料</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>限定资料类型、项目范围或场景边界。</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>服务范围</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>financial</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>财务/金融资料</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>限定资料类型、项目范围或场景边界。</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>服务范围</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>marketing</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>市场宣传资料</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>限定资料类型、项目范围或场景边界。</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>服务范围</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>certified</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>认证/盖章文件</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>限定资料类型、项目范围或场景边界。</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>服务范围</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>confidential</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>保密资料</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>限定资料类型、项目范围或场景边界。</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>服务范围</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>literary_marketing</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>菜单/品牌/文学类资料</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>限定资料类型、项目范围或场景边界。</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>服务范围</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>presentation</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>幻灯片资料</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>限定资料类型、项目范围或场景边界。</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>服务范围</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>native_polishing</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>外籍母语润稿</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>限定资料类型、项目范围或场景边界。</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>服务范围</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>native_translation</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>外籍母语翻译</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>限定资料类型、项目范围或场景边界。</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>服务范围</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>rare_language</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>欧洲稀有语种资料</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>限定资料类型、项目范围或场景边界。</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>服务范围</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>bilingual_foreign</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>双外语翻译</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>限定资料类型、项目范围或场景边界。</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>服务范围</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>formatting</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>输入或排版服务</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>限定资料类型、项目范围或场景边界。</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>客户层级</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>普通客户</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>按客户重要度控制知识适用范围。</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>客户层级</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>key</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>重点客户</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>按客户重要度控制知识适用范围。</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>客户层级</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>strategic</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>战略客户</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>按客户重要度控制知识适用范围。</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>客户层级</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>vip</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>VIP客户</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>按客户重要度控制知识适用范围。</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>风险等级</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>影响审核与发布门禁，报价与限制条件一般为高风险。</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>风险等级</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>影响审核与发布门禁，报价与限制条件一般为高风险。</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>风险等级</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>影响审核与发布门禁，报价与限制条件一般为高风险。</t>
         </is>
       </c>
     </row>

</xml_diff>